<commit_message>
Add pre-merger Two River share count and average cost to cost basis workbook
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_016HFTicFadDMp29ArmvEF6v
</commit_message>
<xml_diff>
--- a/output/OceanFirst_Cost_Basis.xlsx
+++ b/output/OceanFirst_Cost_Basis.xlsx
@@ -28,6 +28,18 @@
     <author>Unknown Author</author>
   </authors>
   <commentList>
+    <comment ref="B16" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">Total row: Two River weighted average cost per share at 12/31/2019 (total investment ÷ total TR shares).</t>
+        </r>
+      </text>
+    </comment>
     <comment ref="B20" authorId="0">
       <text>
         <r>
@@ -129,7 +141,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="48">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="49" uniqueCount="49">
   <si>
     <t xml:space="preserve">Two River Stock Purchase &amp; OceanFirst Merger Cost Basis Analysis</t>
   </si>
@@ -215,10 +227,13 @@
     <t xml:space="preserve">Merger Transfer Summary</t>
   </si>
   <si>
-    <t xml:space="preserve">Total original estimated cost basis</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Total Two River shares before merger</t>
+    <t xml:space="preserve">Total original estimated cost basis (Two River)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Two River shares held at 12/31/2019 (pre-merger)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Two River average cost per share at 12/31/2019</t>
   </si>
   <si>
     <t xml:space="preserve">Cash received at merger</t>
@@ -279,7 +294,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="10">
+  <numFmts count="11">
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="mm/dd/yyyy"/>
     <numFmt numFmtId="166" formatCode="\$#,##0.00;&quot;($&quot;#,##0.00\);\-"/>
@@ -289,7 +304,8 @@
     <numFmt numFmtId="170" formatCode="#,##0.0000"/>
     <numFmt numFmtId="171" formatCode="@"/>
     <numFmt numFmtId="172" formatCode="#,##0"/>
-    <numFmt numFmtId="173" formatCode="0.00%"/>
+    <numFmt numFmtId="173" formatCode="\$#,##0.0000"/>
+    <numFmt numFmtId="174" formatCode="0.00%"/>
   </numFmts>
   <fonts count="14">
     <font>
@@ -479,7 +495,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="44">
+  <cellXfs count="45">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -560,11 +576,15 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="166" fontId="9" fillId="5" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="166" fontId="9" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="167" fontId="9" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="167" fontId="9" fillId="5" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -577,10 +597,6 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="170" fontId="9" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="166" fontId="9" fillId="5" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -628,7 +644,15 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="167" fontId="8" fillId="8" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="9" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="167" fontId="9" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="173" fontId="9" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -636,11 +660,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="173" fontId="8" fillId="8" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="9" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="174" fontId="8" fillId="8" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -953,7 +973,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="A1:M50"/>
+  <dimension ref="A1:M51"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="44"/>
@@ -1608,42 +1628,45 @@
       <c r="A16" s="19" t="s">
         <v>15</v>
       </c>
-      <c r="B16" s="20"/>
-      <c r="C16" s="20" t="n">
+      <c r="B16" s="20" t="n">
+        <f aca="false">IF(D16=0,0,C16/D16)</f>
+        <v>12.4924177431697</v>
+      </c>
+      <c r="C16" s="21" t="n">
         <f aca="false">SUM(C5:C15)</f>
         <v>32492.7785499844</v>
       </c>
-      <c r="D16" s="21" t="n">
+      <c r="D16" s="22" t="n">
         <f aca="false">SUM(D5:D15)</f>
         <v>2601</v>
       </c>
-      <c r="E16" s="22"/>
-      <c r="F16" s="23"/>
-      <c r="G16" s="24" t="n">
+      <c r="E16" s="23"/>
+      <c r="F16" s="24"/>
+      <c r="G16" s="25" t="n">
         <f aca="false">SUM(G5:G15)</f>
         <v>1733.0463</v>
       </c>
-      <c r="H16" s="20" t="n">
+      <c r="H16" s="21" t="n">
         <f aca="false">SUM(H5:H15)</f>
         <v>13980.375</v>
       </c>
-      <c r="I16" s="20" t="n">
+      <c r="I16" s="21" t="n">
         <f aca="false">SUM(I5:I15)</f>
         <v>44262.002502</v>
       </c>
-      <c r="J16" s="20" t="n">
+      <c r="J16" s="21" t="n">
         <f aca="false">SUM(J5:J15)</f>
         <v>25749.5989520156</v>
       </c>
-      <c r="K16" s="20" t="n">
+      <c r="K16" s="21" t="n">
         <f aca="false">SUM(K5:K15)</f>
         <v>12634.8923610538</v>
       </c>
-      <c r="L16" s="25" t="n">
+      <c r="L16" s="20" t="n">
         <f aca="false">SUM(L5:L15)</f>
         <v>31147.2959110382</v>
       </c>
-      <c r="M16" s="25" t="n">
+      <c r="M16" s="20" t="n">
         <f aca="false">IF(G16=0,0,L16/G16)</f>
         <v>17.9725699832937</v>
       </c>
@@ -1748,39 +1771,39 @@
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A31" s="28" t="s">
+      <c r="A31" s="37" t="s">
         <v>29</v>
       </c>
-      <c r="B31" s="37" t="n">
+      <c r="B31" s="38" t="n">
         <f aca="false">D16</f>
         <v>2601</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A32" s="28" t="s">
+      <c r="A32" s="37" t="s">
         <v>30</v>
       </c>
-      <c r="B32" s="36" t="n">
-        <f aca="false">H16</f>
-        <v>13980.375</v>
+      <c r="B32" s="39" t="n">
+        <f aca="false">IF(B31=0,0,B30/B31)</f>
+        <v>12.4924177431697</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="28" t="s">
         <v>31</v>
       </c>
-      <c r="B33" s="38" t="n">
-        <f aca="false">G16</f>
-        <v>1733.0463</v>
+      <c r="B33" s="36" t="n">
+        <f aca="false">H16</f>
+        <v>13980.375</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="28" t="s">
         <v>32</v>
       </c>
-      <c r="B34" s="36" t="n">
-        <f aca="false">I16</f>
-        <v>44262.002502</v>
+      <c r="B34" s="40" t="n">
+        <f aca="false">G16</f>
+        <v>1733.0463</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1788,8 +1811,8 @@
         <v>33</v>
       </c>
       <c r="B35" s="36" t="n">
-        <f aca="false">B32+B34</f>
-        <v>58242.377502</v>
+        <f aca="false">I16</f>
+        <v>44262.002502</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1797,113 +1820,122 @@
         <v>34</v>
       </c>
       <c r="B36" s="36" t="n">
-        <f aca="false">B35-B30</f>
-        <v>25749.5989520156</v>
+        <f aca="false">B33+B35</f>
+        <v>58242.377502</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="28" t="s">
         <v>35</v>
       </c>
-      <c r="B37" s="39" t="n">
-        <f aca="false">IF(B30=0,0,B36/B30)</f>
-        <v>0.792471438304497</v>
+      <c r="B37" s="36" t="n">
+        <f aca="false">B36-B30</f>
+        <v>25749.5989520156</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="28" t="s">
         <v>36</v>
       </c>
-      <c r="B38" s="36" t="n">
-        <f aca="false">K16</f>
-        <v>12634.8923610538</v>
+      <c r="B38" s="41" t="n">
+        <f aca="false">IF(B30=0,0,B37/B30)</f>
+        <v>0.792471438304497</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="28" t="s">
         <v>37</v>
       </c>
-      <c r="B39" s="38" t="n">
-        <f aca="false">G16-$B$24</f>
-        <v>0.0463000000002012</v>
+      <c r="B39" s="36" t="n">
+        <f aca="false">K16</f>
+        <v>12634.8923610538</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="28" t="s">
         <v>38</v>
       </c>
-      <c r="B40" s="36" t="n">
-        <f aca="false">B39*M16</f>
+      <c r="B40" s="40" t="n">
+        <f aca="false">G16-$B$24</f>
+        <v>0.0463000000002012</v>
+      </c>
+    </row>
+    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A41" s="28" t="s">
+        <v>39</v>
+      </c>
+      <c r="B41" s="36" t="n">
+        <f aca="false">B40*M16</f>
         <v>0.832129990230113</v>
       </c>
     </row>
-    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A41" s="40" t="s">
-        <v>39</v>
-      </c>
-      <c r="B41" s="41" t="n">
+    <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A42" s="37" t="s">
+        <v>40</v>
+      </c>
+      <c r="B42" s="42" t="n">
         <f aca="false">$B$24</f>
         <v>1733</v>
       </c>
     </row>
-    <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A42" s="40" t="s">
-        <v>40</v>
-      </c>
-      <c r="B42" s="42" t="n">
-        <f aca="false">L16-B40</f>
+    <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A43" s="37" t="s">
+        <v>41</v>
+      </c>
+      <c r="B43" s="43" t="n">
+        <f aca="false">L16-B41</f>
         <v>31146.4637810479</v>
       </c>
     </row>
-    <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A43" s="40" t="s">
-        <v>41</v>
-      </c>
-      <c r="B43" s="42" t="n">
-        <f aca="false">IF(B41=0,0,B42/B41)</f>
+    <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A44" s="37" t="s">
+        <v>42</v>
+      </c>
+      <c r="B44" s="43" t="n">
+        <f aca="false">IF(B42=0,0,B43/B42)</f>
         <v>17.9725699832937</v>
       </c>
     </row>
-    <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A45" s="27" t="s">
-        <v>42</v>
-      </c>
-      <c r="B45" s="2"/>
-      <c r="C45" s="2"/>
-      <c r="D45" s="2"/>
-      <c r="E45" s="2"/>
-      <c r="F45" s="2"/>
-      <c r="G45" s="2"/>
-      <c r="H45" s="2"/>
-      <c r="I45" s="2"/>
-      <c r="J45" s="2"/>
-      <c r="K45" s="2"/>
-      <c r="L45" s="2"/>
-      <c r="M45" s="2"/>
-    </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A46" s="43" t="s">
+      <c r="A46" s="27" t="s">
         <v>43</v>
       </c>
+      <c r="B46" s="2"/>
+      <c r="C46" s="2"/>
+      <c r="D46" s="2"/>
+      <c r="E46" s="2"/>
+      <c r="F46" s="2"/>
+      <c r="G46" s="2"/>
+      <c r="H46" s="2"/>
+      <c r="I46" s="2"/>
+      <c r="J46" s="2"/>
+      <c r="K46" s="2"/>
+      <c r="L46" s="2"/>
+      <c r="M46" s="2"/>
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A47" s="43" t="s">
+      <c r="A47" s="44" t="s">
         <v>44</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A48" s="43" t="s">
+      <c r="A48" s="44" t="s">
         <v>45</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A49" s="43" t="s">
+      <c r="A49" s="44" t="s">
         <v>46</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A50" s="43" t="s">
+      <c r="A50" s="44" t="s">
         <v>47</v>
+      </c>
+    </row>
+    <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A51" s="44" t="s">
+        <v>48</v>
       </c>
     </row>
   </sheetData>

</xml_diff>